<commit_message>
[auto-snapshot] 2026-04-14 16:00 | onda-hompage | 31 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_nail/강남_네일샵.xlsx
+++ b/naver-place-crawler/results_nail/강남_네일샵.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V438"/>
+  <dimension ref="A1:V445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -41141,34 +41141,26 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>세무사</t>
+          <t>네일아트,네일샵</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>세성세무법인 삼성지점</t>
-        </is>
-      </c>
-      <c r="C437" t="inlineStr">
-        <is>
-          <t>sesung1216@naver.com</t>
-        </is>
-      </c>
+          <t>소금네일</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr"/>
       <c r="D437" t="inlineStr"/>
-      <c r="E437" t="inlineStr">
-        <is>
-          <t>02-515-4642</t>
-        </is>
-      </c>
+      <c r="E437" t="inlineStr"/>
       <c r="F437" t="inlineStr"/>
       <c r="G437" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 봉은사로 454 금탁타워 5층</t>
+          <t>서울특별시 강남구 개포로21길 10 1층</t>
         </is>
       </c>
       <c r="H437" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/sesung1216</t>
+          <t>https://www.instagram.com/sogeum_nail</t>
         </is>
       </c>
       <c r="I437" t="inlineStr">
@@ -41183,7 +41175,7 @@
       </c>
       <c r="K437" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L437" t="inlineStr">
@@ -41199,17 +41191,17 @@
       </c>
       <c r="O437" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P437" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="Q437" t="n">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="R437" t="n">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="S437" t="inlineStr">
         <is>
@@ -41218,12 +41210,12 @@
       </c>
       <c r="T437" t="inlineStr">
         <is>
-          <t>1397509005</t>
+          <t>1003640740</t>
         </is>
       </c>
       <c r="U437" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1397509005</t>
+          <t>https://m.place.naver.com/place/1003640740</t>
         </is>
       </c>
       <c r="V437" t="inlineStr">
@@ -41235,39 +41227,35 @@
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>속눈썹증모,연장</t>
+          <t>네일아트,네일샵</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>워너비뷰티</t>
+          <t>나다움네일</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>doyi2@naver.com</t>
+          <t>onsoo1214@naver.com</t>
         </is>
       </c>
       <c r="D438" t="inlineStr"/>
-      <c r="E438" t="inlineStr">
-        <is>
-          <t>02-552-4043</t>
-        </is>
-      </c>
+      <c r="E438" t="inlineStr"/>
       <c r="F438" t="inlineStr"/>
       <c r="G438" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 삼성로100길 25 2층</t>
+          <t>서울특별시 강남구 도산대로12길 9 3층</t>
         </is>
       </c>
       <c r="H438" t="inlineStr">
         <is>
-          <t>http://pf.kakao.com/_xaxfwTC</t>
+          <t>https://instagram.com/nail_nadaum</t>
         </is>
       </c>
       <c r="I438" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J438" t="inlineStr">
@@ -41288,39 +41276,689 @@
       <c r="M438" t="inlineStr"/>
       <c r="N438" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O438" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P438" t="n">
+        <v>298</v>
+      </c>
+      <c r="Q438" t="n">
+        <v>49</v>
+      </c>
+      <c r="R438" t="n">
+        <v>347</v>
+      </c>
+      <c r="S438" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T438" t="inlineStr">
+        <is>
+          <t>1587252605</t>
+        </is>
+      </c>
+      <c r="U438" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1587252605</t>
+        </is>
+      </c>
+      <c r="V438" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>뷰티인비</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>beauty_inb@naver.com</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr"/>
+      <c r="E439" t="inlineStr"/>
+      <c r="F439" t="inlineStr"/>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 선릉로120길 14 2층</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/beauty_inb</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K439" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L439" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M439" t="inlineStr"/>
+      <c r="N439" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O439" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P439" t="n">
+        <v>412</v>
+      </c>
+      <c r="Q439" t="n">
+        <v>103</v>
+      </c>
+      <c r="R439" t="n">
+        <v>515</v>
+      </c>
+      <c r="S439" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T439" t="inlineStr">
+        <is>
+          <t>1028984231</t>
+        </is>
+      </c>
+      <c r="U439" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1028984231</t>
+        </is>
+      </c>
+      <c r="V439" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>레푸스 강남세곡점</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>segok569@naver.com</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr"/>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>0507-1494-9977</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr"/>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 헌릉로 569 강남리더스프라자 4층 401-1호</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/segok569</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K440" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L440" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M440" t="inlineStr"/>
+      <c r="N440" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O440" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P440" t="n">
+        <v>190</v>
+      </c>
+      <c r="Q440" t="n">
+        <v>480</v>
+      </c>
+      <c r="R440" t="n">
+        <v>670</v>
+      </c>
+      <c r="S440" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T440" t="inlineStr">
+        <is>
+          <t>1486263326</t>
+        </is>
+      </c>
+      <c r="U440" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1486263326</t>
+        </is>
+      </c>
+      <c r="V440" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>엠블랑네일</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>jieun4294@naver.com</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr"/>
+      <c r="E441" t="inlineStr"/>
+      <c r="F441" t="inlineStr"/>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 도산대로85길 30 2층 211호</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_xkRxhxcG</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K441" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L441" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M441" t="inlineStr"/>
+      <c r="N441" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O441" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P441" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q441" t="n">
+        <v>0</v>
+      </c>
+      <c r="R441" t="n">
+        <v>19</v>
+      </c>
+      <c r="S441" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T441" t="inlineStr">
+        <is>
+          <t>1850537636</t>
+        </is>
+      </c>
+      <c r="U441" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1850537636</t>
+        </is>
+      </c>
+      <c r="V441" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>에스제이네일</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>g4um4j4k@naver.com</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr"/>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>0507-1463-4145</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr"/>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 논현로102길 8 101호</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K442" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M442" t="inlineStr"/>
+      <c r="N442" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O442" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P442" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q442" t="n">
+        <v>2</v>
+      </c>
+      <c r="R442" t="n">
+        <v>8</v>
+      </c>
+      <c r="S442" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T442" t="inlineStr">
+        <is>
+          <t>37191892</t>
+        </is>
+      </c>
+      <c r="U442" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/37191892</t>
+        </is>
+      </c>
+      <c r="V442" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>네일앙뜨 강남역점</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>mel_holic@naver.com</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr"/>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>0507-1445-2523</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr"/>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 도곡로3길 19 105호, 106호</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_glsmxj</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K443" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M443" t="inlineStr"/>
+      <c r="N443" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O443" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P443" t="n">
+        <v>533</v>
+      </c>
+      <c r="Q443" t="n">
+        <v>58</v>
+      </c>
+      <c r="R443" t="n">
+        <v>591</v>
+      </c>
+      <c r="S443" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T443" t="inlineStr">
+        <is>
+          <t>1957548139</t>
+        </is>
+      </c>
+      <c r="U443" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1957548139</t>
+        </is>
+      </c>
+      <c r="V443" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>세무사</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>세성세무법인 삼성지점</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>sesung1216@naver.com</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr"/>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>02-515-4642</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr"/>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 봉은사로 454 금탁타워 5층</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/sesung1216</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K444" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M444" t="inlineStr"/>
+      <c r="N444" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O444" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P444" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q444" t="n">
+        <v>41</v>
+      </c>
+      <c r="R444" t="n">
+        <v>41</v>
+      </c>
+      <c r="S444" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T444" t="inlineStr">
+        <is>
+          <t>1397509005</t>
+        </is>
+      </c>
+      <c r="U444" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1397509005</t>
+        </is>
+      </c>
+      <c r="V444" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>속눈썹증모,연장</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>워너비뷰티</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>doyi2@naver.com</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr"/>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>02-552-4043</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr"/>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 삼성로100길 25 2층</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_xaxfwTC</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K445" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L445" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M445" t="inlineStr"/>
+      <c r="N445" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O445" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P445" t="n">
         <v>228</v>
       </c>
-      <c r="Q438" t="n">
+      <c r="Q445" t="n">
         <v>65</v>
       </c>
-      <c r="R438" t="n">
+      <c r="R445" t="n">
         <v>293</v>
       </c>
-      <c r="S438" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="T438" t="inlineStr">
+      <c r="S445" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T445" t="inlineStr">
         <is>
           <t>1523636698</t>
         </is>
       </c>
-      <c r="U438" t="inlineStr">
+      <c r="U445" t="inlineStr">
         <is>
           <t>https://m.place.naver.com/place/1523636698</t>
         </is>
       </c>
-      <c r="V438" t="inlineStr">
+      <c r="V445" t="inlineStr">
         <is>
           <t>2026-04-14</t>
         </is>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-29 16:00 | onda-hompage | 28 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_nail/강남_네일샵.xlsx
+++ b/naver-place-crawler/results_nail/강남_네일샵.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V393"/>
+  <dimension ref="A1:V444"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -36911,34 +36911,34 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>세무사</t>
+          <t>네일아트,네일샵</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>세성세무법인 삼성지점</t>
+          <t>네일산책</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>sesung1216@naver.com</t>
+          <t>nailstroll@naver.com</t>
         </is>
       </c>
       <c r="D392" t="inlineStr"/>
       <c r="E392" t="inlineStr">
         <is>
-          <t>02-515-4642</t>
+          <t>0507-1484-6890</t>
         </is>
       </c>
       <c r="F392" t="inlineStr"/>
       <c r="G392" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 봉은사로 454 금탁타워 5층</t>
+          <t>서울특별시 강남구 봉은사로 471 2층 201-1호</t>
         </is>
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/sesung1216</t>
+          <t>https://www.instagram.com/nailstroll</t>
         </is>
       </c>
       <c r="I392" t="inlineStr">
@@ -36953,7 +36953,7 @@
       </c>
       <c r="K392" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="L392" t="inlineStr">
@@ -36964,22 +36964,22 @@
       <c r="M392" t="inlineStr"/>
       <c r="N392" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="O392" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P392" t="n">
-        <v>0</v>
+        <v>615</v>
       </c>
       <c r="Q392" t="n">
-        <v>44</v>
+        <v>867</v>
       </c>
       <c r="R392" t="n">
-        <v>44</v>
+        <v>1482</v>
       </c>
       <c r="S392" t="inlineStr">
         <is>
@@ -36988,12 +36988,12 @@
       </c>
       <c r="T392" t="inlineStr">
         <is>
-          <t>1397509005</t>
+          <t>1132799547</t>
         </is>
       </c>
       <c r="U392" t="inlineStr">
         <is>
-          <t>https://m.place.naver.com/place/1397509005</t>
+          <t>https://m.place.naver.com/place/1132799547</t>
         </is>
       </c>
       <c r="V392" t="inlineStr">
@@ -37005,35 +37005,39 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>속눈썹증모,연장</t>
+          <t>네일아트,네일샵</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>워너비뷰티</t>
-        </is>
-      </c>
-      <c r="C393" t="inlineStr"/>
+          <t>아캔스탑잇네일</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>everours-@naver.com</t>
+        </is>
+      </c>
       <c r="D393" t="inlineStr"/>
       <c r="E393" t="inlineStr">
         <is>
-          <t>02-552-4043</t>
+          <t>0507-1363-4208</t>
         </is>
       </c>
       <c r="F393" t="inlineStr"/>
       <c r="G393" t="inlineStr">
         <is>
-          <t>서울특별시 강남구 삼성로100길 25 2층</t>
+          <t>서울특별시 강남구 밤고개로 165 근린생활시설 202호</t>
         </is>
       </c>
       <c r="H393" t="inlineStr">
         <is>
-          <t>http://pf.kakao.com/_xaxfwTC</t>
+          <t>https://www.instagram.com/icantstopeatnail</t>
         </is>
       </c>
       <c r="I393" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="J393" t="inlineStr">
@@ -37054,39 +37058,4797 @@
       <c r="M393" t="inlineStr"/>
       <c r="N393" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>X</t>
         </is>
       </c>
       <c r="O393" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="P393" t="n">
+        <v>187</v>
+      </c>
+      <c r="Q393" t="n">
+        <v>10</v>
+      </c>
+      <c r="R393" t="n">
+        <v>197</v>
+      </c>
+      <c r="S393" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T393" t="inlineStr">
+        <is>
+          <t>1351793907</t>
+        </is>
+      </c>
+      <c r="U393" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1351793907</t>
+        </is>
+      </c>
+      <c r="V393" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>앤네일</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>sws0394@naver.com</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr"/>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>0507-1349-8970</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr"/>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 일원로5길 5 1층</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/annnail_55</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M394" t="inlineStr"/>
+      <c r="N394" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O394" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P394" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q394" t="n">
+        <v>60</v>
+      </c>
+      <c r="R394" t="n">
+        <v>75</v>
+      </c>
+      <c r="S394" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T394" t="inlineStr">
+        <is>
+          <t>1303312081</t>
+        </is>
+      </c>
+      <c r="U394" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1303312081</t>
+        </is>
+      </c>
+      <c r="V394" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>네일바이제이</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>minjee1209@naver.com</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr"/>
+      <c r="E395" t="inlineStr"/>
+      <c r="F395" t="inlineStr"/>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 선릉로 328 남서울상가 1층 9호</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nailbyj_j/</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M395" t="inlineStr"/>
+      <c r="N395" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O395" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P395" t="n">
+        <v>288</v>
+      </c>
+      <c r="Q395" t="n">
+        <v>71</v>
+      </c>
+      <c r="R395" t="n">
+        <v>359</v>
+      </c>
+      <c r="S395" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T395" t="inlineStr">
+        <is>
+          <t>37630380</t>
+        </is>
+      </c>
+      <c r="U395" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/37630380</t>
+        </is>
+      </c>
+      <c r="V395" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>르화뷰티</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>writeherh@naver.com</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr"/>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>0507-1400-9350</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr"/>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 남부순환로 2615 1층 122호</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lehwa_beauty</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M396" t="inlineStr"/>
+      <c r="N396" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O396" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P396" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q396" t="n">
+        <v>3</v>
+      </c>
+      <c r="R396" t="n">
+        <v>22</v>
+      </c>
+      <c r="S396" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T396" t="inlineStr">
+        <is>
+          <t>2052556715</t>
+        </is>
+      </c>
+      <c r="U396" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/2052556715</t>
+        </is>
+      </c>
+      <c r="V396" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>제로네일</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr"/>
+      <c r="D397" t="inlineStr"/>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>0507-1422-0014</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr"/>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 압구정로54길 26 3층 제로네일</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>https://pf.kakao.com/_AwIKs</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M397" t="inlineStr"/>
+      <c r="N397" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O397" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P397" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q397" t="n">
+        <v>1</v>
+      </c>
+      <c r="R397" t="n">
+        <v>1</v>
+      </c>
+      <c r="S397" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T397" t="inlineStr">
+        <is>
+          <t>1851003663</t>
+        </is>
+      </c>
+      <c r="U397" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1851003663</t>
+        </is>
+      </c>
+      <c r="V397" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>레푸스 선릉점 인디고네일</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>indigonail@naver.com</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr"/>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>0507-1420-3046</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr"/>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 테헤란로57길 24 1층</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/indigonail</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M398" t="inlineStr"/>
+      <c r="N398" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O398" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P398" t="n">
+        <v>1420</v>
+      </c>
+      <c r="Q398" t="n">
+        <v>682</v>
+      </c>
+      <c r="R398" t="n">
+        <v>2102</v>
+      </c>
+      <c r="S398" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T398" t="inlineStr">
+        <is>
+          <t>35992652</t>
+        </is>
+      </c>
+      <c r="U398" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/35992652</t>
+        </is>
+      </c>
+      <c r="V398" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>바비인형네일&amp;속눈썹</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>4udbfl@naver.com</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr"/>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>0507-1495-5521</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr"/>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 테헤란로1길 44 303호</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/4udbfl</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M399" t="inlineStr"/>
+      <c r="N399" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O399" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P399" t="n">
+        <v>142</v>
+      </c>
+      <c r="Q399" t="n">
+        <v>899</v>
+      </c>
+      <c r="R399" t="n">
+        <v>1041</v>
+      </c>
+      <c r="S399" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T399" t="inlineStr">
+        <is>
+          <t>31676164</t>
+        </is>
+      </c>
+      <c r="U399" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/31676164</t>
+        </is>
+      </c>
+      <c r="V399" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>연네일</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr"/>
+      <c r="D400" t="inlineStr"/>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>02-797-2700</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr"/>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 언주로 118 우성캐릭터199빌딩 130호</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M400" t="inlineStr"/>
+      <c r="N400" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O400" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P400" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q400" t="n">
+        <v>0</v>
+      </c>
+      <c r="R400" t="n">
+        <v>0</v>
+      </c>
+      <c r="S400" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T400" t="inlineStr">
+        <is>
+          <t>20034237</t>
+        </is>
+      </c>
+      <c r="U400" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/20034237</t>
+        </is>
+      </c>
+      <c r="V400" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>도쿄네일 신사점</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>yurinail0610@naver.com</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr"/>
+      <c r="E401" t="inlineStr"/>
+      <c r="F401" t="inlineStr"/>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 논현로149길 65 2층 201호</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/yurinail0610</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M401" t="inlineStr"/>
+      <c r="N401" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O401" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P401" t="n">
+        <v>83</v>
+      </c>
+      <c r="Q401" t="n">
+        <v>59</v>
+      </c>
+      <c r="R401" t="n">
+        <v>142</v>
+      </c>
+      <c r="S401" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T401" t="inlineStr">
+        <is>
+          <t>1676138057</t>
+        </is>
+      </c>
+      <c r="U401" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1676138057</t>
+        </is>
+      </c>
+      <c r="V401" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>더꼼네일</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>kjuuu0716@naver.com</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr"/>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>0507-1375-6412</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr"/>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 테헤란로57길 32 B1</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/the_ccom_nail</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M402" t="inlineStr"/>
+      <c r="N402" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O402" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P402" t="n">
+        <v>128</v>
+      </c>
+      <c r="Q402" t="n">
+        <v>46</v>
+      </c>
+      <c r="R402" t="n">
+        <v>174</v>
+      </c>
+      <c r="S402" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T402" t="inlineStr">
+        <is>
+          <t>1571173388</t>
+        </is>
+      </c>
+      <c r="U402" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1571173388</t>
+        </is>
+      </c>
+      <c r="V402" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>제니스리치 강남역점</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>jennisrich15@naver.com</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr"/>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>0507-1351-3886</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr"/>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 테헤란로4길 6 센트럴 푸르지오 시티 1층</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>https://zero.gongbiz.kr/shop/S000033986</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M403" t="inlineStr"/>
+      <c r="N403" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O403" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P403" t="n">
+        <v>131</v>
+      </c>
+      <c r="Q403" t="n">
+        <v>96</v>
+      </c>
+      <c r="R403" t="n">
+        <v>227</v>
+      </c>
+      <c r="S403" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T403" t="inlineStr">
+        <is>
+          <t>38654257</t>
+        </is>
+      </c>
+      <c r="U403" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/38654257</t>
+        </is>
+      </c>
+      <c r="V403" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>참살롱</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>charm_salon@naver.com</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr"/>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>0507-1340-9017</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr"/>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 자곡로 202 1층 109호</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/CHAM_salon_official</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M404" t="inlineStr"/>
+      <c r="N404" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O404" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P404" t="n">
+        <v>169</v>
+      </c>
+      <c r="Q404" t="n">
+        <v>0</v>
+      </c>
+      <c r="R404" t="n">
+        <v>169</v>
+      </c>
+      <c r="S404" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T404" t="inlineStr">
+        <is>
+          <t>1081725462</t>
+        </is>
+      </c>
+      <c r="U404" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1081725462</t>
+        </is>
+      </c>
+      <c r="V404" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>더파이브센스</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>kmy000403@naver.com</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr"/>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>0507-1380-4121</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr"/>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 논현로114길 11 해광빌딩 1층 더파이브센스(The5Sneses)</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com//the5senses_</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M405" t="inlineStr"/>
+      <c r="N405" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O405" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P405" t="n">
+        <v>180</v>
+      </c>
+      <c r="Q405" t="n">
+        <v>145</v>
+      </c>
+      <c r="R405" t="n">
+        <v>325</v>
+      </c>
+      <c r="S405" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T405" t="inlineStr">
+        <is>
+          <t>1213490829</t>
+        </is>
+      </c>
+      <c r="U405" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1213490829</t>
+        </is>
+      </c>
+      <c r="V405" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>내일디디</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>black585@naver.com</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr"/>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>0507-1341-5722</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr"/>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 압구정로50길 18 6층 601호</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/tomorrow.dd_</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K406" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M406" t="inlineStr"/>
+      <c r="N406" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O406" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P406" t="n">
+        <v>379</v>
+      </c>
+      <c r="Q406" t="n">
+        <v>601</v>
+      </c>
+      <c r="R406" t="n">
+        <v>980</v>
+      </c>
+      <c r="S406" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T406" t="inlineStr">
+        <is>
+          <t>1941401558</t>
+        </is>
+      </c>
+      <c r="U406" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1941401558</t>
+        </is>
+      </c>
+      <c r="V406" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>신사동 네일 더누크룸</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>mmming112@naver.com</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr"/>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>0507-1477-8027</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr"/>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 압구정로14길 35 2층 202호</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_KWVnn</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K407" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M407" t="inlineStr"/>
+      <c r="N407" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O407" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P407" t="n">
+        <v>56</v>
+      </c>
+      <c r="Q407" t="n">
+        <v>9</v>
+      </c>
+      <c r="R407" t="n">
+        <v>65</v>
+      </c>
+      <c r="S407" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T407" t="inlineStr">
+        <is>
+          <t>1616156850</t>
+        </is>
+      </c>
+      <c r="U407" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1616156850</t>
+        </is>
+      </c>
+      <c r="V407" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>강남네일맑음</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>s1514@naver.com</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr"/>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>0507-1410-3143</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr"/>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 강남대로78길 24 3층 강남네일맑음</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>https://pf.kakao.com/_xmzLxfxb</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K408" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M408" t="inlineStr"/>
+      <c r="N408" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O408" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P408" t="n">
+        <v>2526</v>
+      </c>
+      <c r="Q408" t="n">
+        <v>360</v>
+      </c>
+      <c r="R408" t="n">
+        <v>2886</v>
+      </c>
+      <c r="S408" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T408" t="inlineStr">
+        <is>
+          <t>37700060</t>
+        </is>
+      </c>
+      <c r="U408" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/37700060</t>
+        </is>
+      </c>
+      <c r="V408" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>베릴네일</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>s2binini@naver.com</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr"/>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>0507-1407-5026</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr"/>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 언주로93길 29 4층 401호</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/berylnail_</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K409" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M409" t="inlineStr"/>
+      <c r="N409" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O409" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P409" t="n">
+        <v>122</v>
+      </c>
+      <c r="Q409" t="n">
+        <v>11</v>
+      </c>
+      <c r="R409" t="n">
+        <v>133</v>
+      </c>
+      <c r="S409" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T409" t="inlineStr">
+        <is>
+          <t>1208197127</t>
+        </is>
+      </c>
+      <c r="U409" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1208197127</t>
+        </is>
+      </c>
+      <c r="V409" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>핀업네일</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>mirabia0714@naver.com</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr"/>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>02-515-8087</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr"/>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 도산대로62길 15 1층 핀업네일</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>https://instagram.com/pinupnail_?igshid=OGQ5ZDc2ODk2ZA==</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K410" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M410" t="inlineStr"/>
+      <c r="N410" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O410" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P410" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q410" t="n">
+        <v>4</v>
+      </c>
+      <c r="R410" t="n">
+        <v>31</v>
+      </c>
+      <c r="S410" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T410" t="inlineStr">
+        <is>
+          <t>1597938714</t>
+        </is>
+      </c>
+      <c r="U410" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1597938714</t>
+        </is>
+      </c>
+      <c r="V410" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>벨로네일</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>allprettylove@naver.com</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr"/>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>0507-1402-0155</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr"/>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 양재대로33길 21 1층 102호</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>http://instagram.com/nail_h4845</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K411" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M411" t="inlineStr"/>
+      <c r="N411" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O411" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P411" t="n">
+        <v>99</v>
+      </c>
+      <c r="Q411" t="n">
+        <v>16</v>
+      </c>
+      <c r="R411" t="n">
+        <v>115</v>
+      </c>
+      <c r="S411" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T411" t="inlineStr">
+        <is>
+          <t>1046516068</t>
+        </is>
+      </c>
+      <c r="U411" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1046516068</t>
+        </is>
+      </c>
+      <c r="V411" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>홍혜선프로네일</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>wootak1626@naver.com</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr"/>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>0507-1389-2368</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr"/>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 학동로38길 40 1층 101호</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/honghyesun_pronail/</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K412" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M412" t="inlineStr"/>
+      <c r="N412" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O412" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P412" t="n">
+        <v>399</v>
+      </c>
+      <c r="Q412" t="n">
+        <v>133</v>
+      </c>
+      <c r="R412" t="n">
+        <v>532</v>
+      </c>
+      <c r="S412" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T412" t="inlineStr">
+        <is>
+          <t>1488876783</t>
+        </is>
+      </c>
+      <c r="U412" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1488876783</t>
+        </is>
+      </c>
+      <c r="V412" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>제이네일</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>rhkdmswl@naver.com</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr"/>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>0507-1362-6427</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr"/>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 선릉로 206 동부센트레빌 상가 1층 117호</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>https://homefine2470.mycafe24.com/</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K413" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M413" t="inlineStr"/>
+      <c r="N413" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O413" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P413" t="n">
+        <v>33</v>
+      </c>
+      <c r="Q413" t="n">
+        <v>3</v>
+      </c>
+      <c r="R413" t="n">
+        <v>36</v>
+      </c>
+      <c r="S413" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T413" t="inlineStr">
+        <is>
+          <t>2070234334</t>
+        </is>
+      </c>
+      <c r="U413" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/2070234334</t>
+        </is>
+      </c>
+      <c r="V413" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>네일 움뷰티</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>myvely1@naver.com</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr"/>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>0507-1336-2648</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr"/>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 학동로34길 20 3층</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/myvely1</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K414" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L414" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M414" t="inlineStr"/>
+      <c r="N414" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O414" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P414" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q414" t="n">
+        <v>29</v>
+      </c>
+      <c r="R414" t="n">
+        <v>48</v>
+      </c>
+      <c r="S414" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T414" t="inlineStr">
+        <is>
+          <t>1674089540</t>
+        </is>
+      </c>
+      <c r="U414" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1674089540</t>
+        </is>
+      </c>
+      <c r="V414" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>에드민 네일</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>addmin3411@naver.com</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr"/>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>0507-1300-3411</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr"/>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 강남대로120길 31 1층 에드민네일</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/addmin_nail/</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K415" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L415" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M415" t="inlineStr"/>
+      <c r="N415" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O415" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P415" t="n">
+        <v>240</v>
+      </c>
+      <c r="Q415" t="n">
+        <v>48</v>
+      </c>
+      <c r="R415" t="n">
+        <v>288</v>
+      </c>
+      <c r="S415" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T415" t="inlineStr">
+        <is>
+          <t>1706496056</t>
+        </is>
+      </c>
+      <c r="U415" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1706496056</t>
+        </is>
+      </c>
+      <c r="V415" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>오늘네일</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>todaynnail@naver.com</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr"/>
+      <c r="E416" t="inlineStr"/>
+      <c r="F416" t="inlineStr"/>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 개포로82길 13-11 2층 204호 오늘네일</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/todaynnail</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K416" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L416" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M416" t="inlineStr"/>
+      <c r="N416" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O416" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P416" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q416" t="n">
+        <v>28</v>
+      </c>
+      <c r="R416" t="n">
+        <v>31</v>
+      </c>
+      <c r="S416" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T416" t="inlineStr">
+        <is>
+          <t>1213126581</t>
+        </is>
+      </c>
+      <c r="U416" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1213126581</t>
+        </is>
+      </c>
+      <c r="V416" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>초승달네일</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>miwoomiwoo27@naver.com</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr"/>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>0507-1357-0944</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr"/>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 삼성로71길 37 지상1층 102호</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nailcrescent</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K417" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L417" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M417" t="inlineStr"/>
+      <c r="N417" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O417" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P417" t="n">
+        <v>139</v>
+      </c>
+      <c r="Q417" t="n">
+        <v>3</v>
+      </c>
+      <c r="R417" t="n">
+        <v>142</v>
+      </c>
+      <c r="S417" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T417" t="inlineStr">
+        <is>
+          <t>1925396402</t>
+        </is>
+      </c>
+      <c r="U417" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1925396402</t>
+        </is>
+      </c>
+      <c r="V417" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>네일포시즌 풋풋한리쌤 역삼점</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>footfoot4@naver.com</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr"/>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>02-6953-3236</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr"/>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 봉은사로 206 2층</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/footfoot4</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K418" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L418" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M418" t="inlineStr"/>
+      <c r="N418" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O418" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P418" t="n">
+        <v>2099</v>
+      </c>
+      <c r="Q418" t="n">
+        <v>245</v>
+      </c>
+      <c r="R418" t="n">
+        <v>2344</v>
+      </c>
+      <c r="S418" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T418" t="inlineStr">
+        <is>
+          <t>1556154058</t>
+        </is>
+      </c>
+      <c r="U418" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1556154058</t>
+        </is>
+      </c>
+      <c r="V418" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>글로이네일</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>sh_0503@naver.com</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr"/>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>0507-1406-1721</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr"/>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 헌릉로571길 9 1층 106호 글로이네일</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/glowwy_nail</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K419" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M419" t="inlineStr"/>
+      <c r="N419" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O419" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P419" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q419" t="n">
+        <v>1</v>
+      </c>
+      <c r="R419" t="n">
+        <v>31</v>
+      </c>
+      <c r="S419" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T419" t="inlineStr">
+        <is>
+          <t>2075735615</t>
+        </is>
+      </c>
+      <c r="U419" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/2075735615</t>
+        </is>
+      </c>
+      <c r="V419" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>투떰즈업네일</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>2thumbsup-nail@naver.com</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr"/>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>0507-1381-9779</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr"/>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 도산대로 158 101호</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/2thumbsup_nail</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K420" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L420" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M420" t="inlineStr"/>
+      <c r="N420" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O420" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P420" t="n">
+        <v>121</v>
+      </c>
+      <c r="Q420" t="n">
+        <v>70</v>
+      </c>
+      <c r="R420" t="n">
+        <v>191</v>
+      </c>
+      <c r="S420" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T420" t="inlineStr">
+        <is>
+          <t>1370289480</t>
+        </is>
+      </c>
+      <c r="U420" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1370289480</t>
+        </is>
+      </c>
+      <c r="V420" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>레이네일 앤 풋스파</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>yoo06007@naver.com</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr"/>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>0507-1379-0569</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr"/>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 삼성로 11 디에이치아너힐즈 상가 B108</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>http://instagram.com/leynail_</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K421" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L421" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M421" t="inlineStr"/>
+      <c r="N421" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O421" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P421" t="n">
+        <v>67</v>
+      </c>
+      <c r="Q421" t="n">
+        <v>123</v>
+      </c>
+      <c r="R421" t="n">
+        <v>190</v>
+      </c>
+      <c r="S421" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T421" t="inlineStr">
+        <is>
+          <t>972598699</t>
+        </is>
+      </c>
+      <c r="U421" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/972598699</t>
+        </is>
+      </c>
+      <c r="V421" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>림네일*</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>freshgang@naver.com</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr"/>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>0507-1323-5549</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr"/>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 언주로 118 오피스텔건물</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K422" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L422" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M422" t="inlineStr"/>
+      <c r="N422" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O422" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P422" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q422" t="n">
+        <v>1</v>
+      </c>
+      <c r="R422" t="n">
+        <v>1</v>
+      </c>
+      <c r="S422" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T422" t="inlineStr">
+        <is>
+          <t>1109281431</t>
+        </is>
+      </c>
+      <c r="U422" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1109281431</t>
+        </is>
+      </c>
+      <c r="V422" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>아이리스네일</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>baaa123@naver.com</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr"/>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>0507-1412-8911</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr"/>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 역삼로63길 20 2층 아이리스네일</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K423" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L423" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M423" t="inlineStr"/>
+      <c r="N423" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O423" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P423" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q423" t="n">
+        <v>20</v>
+      </c>
+      <c r="R423" t="n">
+        <v>22</v>
+      </c>
+      <c r="S423" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T423" t="inlineStr">
+        <is>
+          <t>1711649989</t>
+        </is>
+      </c>
+      <c r="U423" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1711649989</t>
+        </is>
+      </c>
+      <c r="V423" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>포쉬네일 하이푸스 가로수길점</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>6607144@naver.com</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr"/>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>0507-1374-6141</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr"/>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 가로수길 16 3층 포쉬네일 하이푸스 가로수길점</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/hifuss_garosugil</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K424" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M424" t="inlineStr"/>
+      <c r="N424" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O424" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P424" t="n">
+        <v>1335</v>
+      </c>
+      <c r="Q424" t="n">
+        <v>552</v>
+      </c>
+      <c r="R424" t="n">
+        <v>1887</v>
+      </c>
+      <c r="S424" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T424" t="inlineStr">
+        <is>
+          <t>20378592</t>
+        </is>
+      </c>
+      <c r="U424" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/20378592</t>
+        </is>
+      </c>
+      <c r="V424" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>임스네일</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>jkhsdm@naver.com</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr"/>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>0507-1483-3322</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr"/>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 도곡로25길 31 1층</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/lim.s_nail23</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K425" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M425" t="inlineStr"/>
+      <c r="N425" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O425" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P425" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q425" t="n">
+        <v>4</v>
+      </c>
+      <c r="R425" t="n">
+        <v>9</v>
+      </c>
+      <c r="S425" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T425" t="inlineStr">
+        <is>
+          <t>1409642751</t>
+        </is>
+      </c>
+      <c r="U425" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1409642751</t>
+        </is>
+      </c>
+      <c r="V425" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>네일도예쁨</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>555__555@naver.com</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr"/>
+      <c r="E426" t="inlineStr"/>
+      <c r="F426" t="inlineStr"/>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 도곡로93길 12 래미안하이스턴상가 1층 102호 네일도예쁨</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K426" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M426" t="inlineStr"/>
+      <c r="N426" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O426" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P426" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q426" t="n">
+        <v>10</v>
+      </c>
+      <c r="R426" t="n">
+        <v>25</v>
+      </c>
+      <c r="S426" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T426" t="inlineStr">
+        <is>
+          <t>1026259823</t>
+        </is>
+      </c>
+      <c r="U426" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1026259823</t>
+        </is>
+      </c>
+      <c r="V426" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>보이니 네일</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>love_hpness@naver.com</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr"/>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>0507-1362-3065</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr"/>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 압구정로10길 30-8 4층 (마사타코 건물로 들어오세요)</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/BOINEE_NAIL</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K427" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M427" t="inlineStr"/>
+      <c r="N427" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O427" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P427" t="n">
+        <v>180</v>
+      </c>
+      <c r="Q427" t="n">
+        <v>11</v>
+      </c>
+      <c r="R427" t="n">
+        <v>191</v>
+      </c>
+      <c r="S427" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T427" t="inlineStr">
+        <is>
+          <t>1147038913</t>
+        </is>
+      </c>
+      <c r="U427" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1147038913</t>
+        </is>
+      </c>
+      <c r="V427" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>네일슈슈</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>brilliant14694@naver.com</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr"/>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>0507-1444-1395</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr"/>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 테헤란로52길 16 테헤란아이파크상가4호</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nail_shushu/</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K428" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M428" t="inlineStr"/>
+      <c r="N428" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O428" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P428" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q428" t="n">
+        <v>15</v>
+      </c>
+      <c r="R428" t="n">
+        <v>15</v>
+      </c>
+      <c r="S428" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T428" t="inlineStr">
+        <is>
+          <t>38264509</t>
+        </is>
+      </c>
+      <c r="U428" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/38264509</t>
+        </is>
+      </c>
+      <c r="V428" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>팔색조네일</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>3157520@naver.com</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr"/>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>0507-1494-2781</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr"/>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 학동로4길 10 3층 304호 팔색조네일</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/8colornail</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K429" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M429" t="inlineStr"/>
+      <c r="N429" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O429" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P429" t="n">
+        <v>68</v>
+      </c>
+      <c r="Q429" t="n">
+        <v>136</v>
+      </c>
+      <c r="R429" t="n">
+        <v>204</v>
+      </c>
+      <c r="S429" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T429" t="inlineStr">
+        <is>
+          <t>1383221614</t>
+        </is>
+      </c>
+      <c r="U429" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1383221614</t>
+        </is>
+      </c>
+      <c r="V429" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>끌레르 네일</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>dunggmi@naver.com</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr"/>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>02-577-4359</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr"/>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 선릉로 8 래미안블레스티지 근린생활시설 지하1층 28-1호</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K430" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M430" t="inlineStr"/>
+      <c r="N430" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O430" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P430" t="n">
+        <v>286</v>
+      </c>
+      <c r="Q430" t="n">
+        <v>7</v>
+      </c>
+      <c r="R430" t="n">
+        <v>293</v>
+      </c>
+      <c r="S430" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T430" t="inlineStr">
+        <is>
+          <t>1425622508</t>
+        </is>
+      </c>
+      <c r="U430" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1425622508</t>
+        </is>
+      </c>
+      <c r="V430" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>쥬이네일</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>zuy0ung@naver.com</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr"/>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>0507-1311-5621</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr"/>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 일원로5길 54 1층</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/juee_nail?igsh=ZGdiY2g5a2FyemRu&amp;utm_source=qr</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K431" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M431" t="inlineStr"/>
+      <c r="N431" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O431" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P431" t="n">
+        <v>202</v>
+      </c>
+      <c r="Q431" t="n">
+        <v>83</v>
+      </c>
+      <c r="R431" t="n">
+        <v>285</v>
+      </c>
+      <c r="S431" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T431" t="inlineStr">
+        <is>
+          <t>1791943614</t>
+        </is>
+      </c>
+      <c r="U431" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1791943614</t>
+        </is>
+      </c>
+      <c r="V431" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>빼꼼네일&amp;뷰티</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>hemni0228@naver.com</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr"/>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>0507-1305-8739</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr"/>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 선릉로126길 14-12 1층 빼꼼네일</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_LAMab</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K432" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M432" t="inlineStr"/>
+      <c r="N432" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O432" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P432" t="n">
+        <v>517</v>
+      </c>
+      <c r="Q432" t="n">
+        <v>50</v>
+      </c>
+      <c r="R432" t="n">
+        <v>567</v>
+      </c>
+      <c r="S432" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T432" t="inlineStr">
+        <is>
+          <t>1769410350</t>
+        </is>
+      </c>
+      <c r="U432" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1769410350</t>
+        </is>
+      </c>
+      <c r="V432" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>에이치인 네일</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>92_10_13@naver.com</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr"/>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>0507-1313-4230</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr"/>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 삼성로103길 22 1층 1-2호</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>http://www.instagram.com/h.in_nail</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K433" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M433" t="inlineStr"/>
+      <c r="N433" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O433" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P433" t="n">
+        <v>55</v>
+      </c>
+      <c r="Q433" t="n">
+        <v>6</v>
+      </c>
+      <c r="R433" t="n">
+        <v>61</v>
+      </c>
+      <c r="S433" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T433" t="inlineStr">
+        <is>
+          <t>1132309657</t>
+        </is>
+      </c>
+      <c r="U433" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1132309657</t>
+        </is>
+      </c>
+      <c r="V433" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>언드네일</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>kmj5_5@naver.com</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr"/>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>0507-1349-0237</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr"/>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 학동로45길 3-4 4층</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_xoxeKNn</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K434" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L434" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M434" t="inlineStr"/>
+      <c r="N434" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O434" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P434" t="n">
+        <v>49</v>
+      </c>
+      <c r="Q434" t="n">
+        <v>1</v>
+      </c>
+      <c r="R434" t="n">
+        <v>50</v>
+      </c>
+      <c r="S434" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T434" t="inlineStr">
+        <is>
+          <t>2082058115</t>
+        </is>
+      </c>
+      <c r="U434" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/2082058115</t>
+        </is>
+      </c>
+      <c r="V434" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>네일원스튜디오</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>pear0406@naver.com</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr"/>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>0507-1447-1054</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr"/>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 압구정로46길 35 B1층 고바이씬 NAIL.1STUDIO</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/nail.1studio__?igsh=MXB1ajdoNmV3aTIzag==</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K435" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L435" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M435" t="inlineStr"/>
+      <c r="N435" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O435" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P435" t="n">
+        <v>217</v>
+      </c>
+      <c r="Q435" t="n">
+        <v>10</v>
+      </c>
+      <c r="R435" t="n">
+        <v>227</v>
+      </c>
+      <c r="S435" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T435" t="inlineStr">
+        <is>
+          <t>1311074001</t>
+        </is>
+      </c>
+      <c r="U435" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1311074001</t>
+        </is>
+      </c>
+      <c r="V435" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>네일20 선릉본점</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>gjbnxouijl315@naver.com</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr"/>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>0507-1304-4157</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr"/>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 테헤란로64길 25 5층</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_vkPsxj</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K436" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L436" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M436" t="inlineStr"/>
+      <c r="N436" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O436" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P436" t="n">
+        <v>1383</v>
+      </c>
+      <c r="Q436" t="n">
+        <v>728</v>
+      </c>
+      <c r="R436" t="n">
+        <v>2111</v>
+      </c>
+      <c r="S436" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T436" t="inlineStr">
+        <is>
+          <t>1226520921</t>
+        </is>
+      </c>
+      <c r="U436" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1226520921</t>
+        </is>
+      </c>
+      <c r="V436" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>미쥬네일 강남신논현점</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>ksmko2026@naver.com</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr"/>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>0507-1446-0689</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr"/>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 봉은사로2길 13 3층</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_PxehYs/chat</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K437" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M437" t="inlineStr"/>
+      <c r="N437" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O437" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P437" t="n">
+        <v>694</v>
+      </c>
+      <c r="Q437" t="n">
+        <v>82</v>
+      </c>
+      <c r="R437" t="n">
+        <v>776</v>
+      </c>
+      <c r="S437" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T437" t="inlineStr">
+        <is>
+          <t>1375175853</t>
+        </is>
+      </c>
+      <c r="U437" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1375175853</t>
+        </is>
+      </c>
+      <c r="V437" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>whyznail</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>whyznail@naver.com</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr"/>
+      <c r="E438" t="inlineStr"/>
+      <c r="F438" t="inlineStr"/>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 선릉로146길 11</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/whyznail</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K438" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M438" t="inlineStr"/>
+      <c r="N438" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O438" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P438" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q438" t="n">
+        <v>0</v>
+      </c>
+      <c r="R438" t="n">
+        <v>0</v>
+      </c>
+      <c r="S438" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T438" t="inlineStr">
+        <is>
+          <t>36771867</t>
+        </is>
+      </c>
+      <c r="U438" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/36771867</t>
+        </is>
+      </c>
+      <c r="V438" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>레푸스 강남세곡점</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>segok569@naver.com</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr"/>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>0507-1494-9977</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr"/>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 헌릉로 569 강남리더스프라자 4층 401-1호</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/segok569</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K439" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L439" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M439" t="inlineStr"/>
+      <c r="N439" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O439" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P439" t="n">
+        <v>191</v>
+      </c>
+      <c r="Q439" t="n">
+        <v>483</v>
+      </c>
+      <c r="R439" t="n">
+        <v>674</v>
+      </c>
+      <c r="S439" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T439" t="inlineStr">
+        <is>
+          <t>1486263326</t>
+        </is>
+      </c>
+      <c r="U439" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1486263326</t>
+        </is>
+      </c>
+      <c r="V439" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>뷰티블룸</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>ksi6439@naver.com</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr"/>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>070-4115-0656</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr"/>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 학동로 342 sk허브 지하1층 117호</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>http://instagram.com/b.bloom_nail</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K440" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L440" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M440" t="inlineStr"/>
+      <c r="N440" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O440" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P440" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q440" t="n">
+        <v>7</v>
+      </c>
+      <c r="R440" t="n">
+        <v>18</v>
+      </c>
+      <c r="S440" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T440" t="inlineStr">
+        <is>
+          <t>746435071</t>
+        </is>
+      </c>
+      <c r="U440" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/746435071</t>
+        </is>
+      </c>
+      <c r="V440" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>네일감성</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>gab316@naver.com</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr"/>
+      <c r="E441" t="inlineStr"/>
+      <c r="F441" t="inlineStr"/>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 선릉로130길 20 래미안삼성2차상가 2층 네일감성</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/_nailbbo</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K441" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L441" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M441" t="inlineStr"/>
+      <c r="N441" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O441" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P441" t="n">
+        <v>52</v>
+      </c>
+      <c r="Q441" t="n">
+        <v>1</v>
+      </c>
+      <c r="R441" t="n">
+        <v>53</v>
+      </c>
+      <c r="S441" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T441" t="inlineStr">
+        <is>
+          <t>1962553293</t>
+        </is>
+      </c>
+      <c r="U441" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1962553293</t>
+        </is>
+      </c>
+      <c r="V441" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>네일아트,네일샵</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>플디아네일</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>syonnyshinny0_0@naver.com</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr"/>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>0507-1486-2397</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr"/>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 학동로55길 12-7 102호</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_xhtxaKn</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K442" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M442" t="inlineStr"/>
+      <c r="N442" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O442" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="P442" t="n">
+        <v>145</v>
+      </c>
+      <c r="Q442" t="n">
+        <v>22</v>
+      </c>
+      <c r="R442" t="n">
+        <v>167</v>
+      </c>
+      <c r="S442" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T442" t="inlineStr">
+        <is>
+          <t>1925563003</t>
+        </is>
+      </c>
+      <c r="U442" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1925563003</t>
+        </is>
+      </c>
+      <c r="V442" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>세무사</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>세성세무법인 삼성지점</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>sesung1216@naver.com</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr"/>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>02-515-4642</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr"/>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 봉은사로 454 금탁타워 5층</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>https://blog.naver.com/sesung1216</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K443" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M443" t="inlineStr"/>
+      <c r="N443" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="O443" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P443" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q443" t="n">
+        <v>44</v>
+      </c>
+      <c r="R443" t="n">
+        <v>44</v>
+      </c>
+      <c r="S443" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T443" t="inlineStr">
+        <is>
+          <t>1397509005</t>
+        </is>
+      </c>
+      <c r="U443" t="inlineStr">
+        <is>
+          <t>https://m.place.naver.com/place/1397509005</t>
+        </is>
+      </c>
+      <c r="V443" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>속눈썹증모,연장</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>워너비뷰티</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr"/>
+      <c r="D444" t="inlineStr"/>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>02-552-4043</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr"/>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>서울특별시 강남구 삼성로100길 25 2층</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>http://pf.kakao.com/_xaxfwTC</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="K444" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M444" t="inlineStr"/>
+      <c r="N444" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="O444" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P444" t="n">
         <v>230</v>
       </c>
-      <c r="Q393" t="n">
+      <c r="Q444" t="n">
         <v>66</v>
       </c>
-      <c r="R393" t="n">
+      <c r="R444" t="n">
         <v>296</v>
       </c>
-      <c r="S393" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="T393" t="inlineStr">
+      <c r="S444" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="T444" t="inlineStr">
         <is>
           <t>1523636698</t>
         </is>
       </c>
-      <c r="U393" t="inlineStr">
+      <c r="U444" t="inlineStr">
         <is>
           <t>https://m.place.naver.com/place/1523636698</t>
         </is>
       </c>
-      <c r="V393" t="inlineStr">
+      <c r="V444" t="inlineStr">
         <is>
           <t>2026-04-29</t>
         </is>

</xml_diff>